<commit_message>
Fill 1 and 10 Oct as A, leave days after 22 Oct blank
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LsGdck9uUBqMn7Bw6wMhA5
</commit_message>
<xml_diff>
--- a/Personel_Devam_Cizelgesi_Ekim_2026_FURKAN_BAYKUSAK.xlsx
+++ b/Personel_Devam_Cizelgesi_Ekim_2026_FURKAN_BAYKUSAK.xlsx
@@ -1196,13 +1196,21 @@
       <c r="B15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="28" t="n"/>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="6" t="n"/>
-      <c r="I15" s="28" t="n"/>
+      <c r="I15" s="28" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="7" t="n"/>
     </row>
@@ -1386,13 +1394,21 @@
       <c r="B24" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="C24" s="28" t="n"/>
+      <c r="C24" s="28" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
       <c r="D24" s="6" t="n"/>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="n"/>
       <c r="H24" s="6" t="n"/>
-      <c r="I24" s="28" t="n"/>
+      <c r="I24" s="28" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
       <c r="J24" s="9" t="n"/>
       <c r="K24" s="10" t="n"/>
     </row>
@@ -1664,21 +1680,13 @@
       <c r="B37" s="8" t="n">
         <v>23</v>
       </c>
-      <c r="C37" s="28" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
+      <c r="C37" s="28" t="n"/>
       <c r="D37" s="6" t="n"/>
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="n"/>
       <c r="G37" s="6" t="n"/>
       <c r="H37" s="6" t="n"/>
-      <c r="I37" s="28" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
+      <c r="I37" s="28" t="n"/>
       <c r="J37" s="9" t="n"/>
       <c r="K37" s="10" t="n"/>
     </row>
@@ -1686,21 +1694,13 @@
       <c r="B38" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="C38" s="28" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
+      <c r="C38" s="28" t="n"/>
       <c r="D38" s="6" t="n"/>
       <c r="E38" s="6" t="n"/>
       <c r="F38" s="6" t="n"/>
       <c r="G38" s="6" t="n"/>
       <c r="H38" s="6" t="n"/>
-      <c r="I38" s="28" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
+      <c r="I38" s="28" t="n"/>
       <c r="J38" s="9" t="n"/>
       <c r="K38" s="10" t="n"/>
     </row>
@@ -1708,21 +1708,13 @@
       <c r="B39" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="C39" s="28" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
+      <c r="C39" s="28" t="n"/>
       <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n"/>
       <c r="G39" s="6" t="n"/>
       <c r="H39" s="6" t="n"/>
-      <c r="I39" s="28" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
+      <c r="I39" s="28" t="n"/>
       <c r="J39" s="9" t="n"/>
       <c r="K39" s="10" t="n"/>
     </row>

</xml_diff>